<commit_message>
correccion de codigo y validacion de campos requeridos
</commit_message>
<xml_diff>
--- a/data/ejemplo_inventario_ips.xlsx
+++ b/data/ejemplo_inventario_ips.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>452536958T</t>
+          <t>SERVICIO-DEMO-A</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
@@ -655,7 +655,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>253644789T</t>
+          <t>SERVICIO-DEMO-B</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
@@ -693,7 +693,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>253658749T</t>
+          <t>SERVICIO-DEMO-C</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
@@ -731,7 +731,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>122025745T</t>
+          <t>SERVICIO-DEMO-D</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">

</xml_diff>